<commit_message>
Update NY gaming data - Thu Sep 17 17:20:43 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_analysis.xlsx
+++ b/ny_gaming_analysis.xlsx
@@ -493,28 +493,28 @@
         <v>35436082</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>36284766</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>216744126</v>
       </c>
       <c r="F2" t="n">
-        <v>224469222</v>
+        <v>224469223</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>60516979</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>10420724</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>7510657</v>
       </c>
       <c r="K2" t="n">
-        <v>263117002</v>
+        <v>594594255</v>
       </c>
     </row>
     <row r="3">
@@ -9139,28 +9139,28 @@
         <v>966974</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1130590</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>4743263</v>
       </c>
       <c r="F2" t="n">
-        <v>8347252.089999981</v>
+        <v>8347252</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>642600</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>608148</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>420192</v>
       </c>
       <c r="K2" t="n">
-        <v>9418255.089999981</v>
+        <v>16963048</v>
       </c>
     </row>
     <row r="3">
@@ -17784,17 +17784,27 @@
       <c r="C2" s="2" t="n">
         <v>0.02728783616653782</v>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>0.03115880642581518</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.02188415938893772</v>
+      </c>
       <c r="F2" s="2" t="n">
-        <v>0.03718662191469609</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+        <v>0.03718662134808566</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.0106185075761961</v>
+      </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" s="2" t="n">
+        <v>0.05835947675036782</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0.05594610431550795</v>
+      </c>
       <c r="K2" s="2" t="n">
-        <v>0.03579493160232945</v>
+        <v>0.02852877883927755</v>
       </c>
     </row>
     <row r="3">
@@ -26151,26 +26161,26 @@
         <v>0.1072158051909604</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1</v>
+        <v>0.08453915426801406</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1</v>
+        <v>0.07104311570147237</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.2824596302339613</v>
+        <v>0.2824596359472595</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.08246389845103475</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
-        <v>-1</v>
+        <v>0.003940046399617314</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.3563374433577221</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.5070743237183399</v>
+        <v>0.1139180403821447</v>
       </c>
     </row>
     <row r="3">
@@ -33601,26 +33611,26 @@
         <v>-0.6132223127527672</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.5642684647977758</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.7645204580808593</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-0.6535737911814852</v>
+        <v>-0.6535737949166487</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.8838066083409352</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.4230866648768997</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.4056337151570532</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.834368666615245</v>
+        <v>-0.7016844169475974</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Update NY gaming data - Thu Sep 24 20:20:41 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_analysis.xlsx
+++ b/ny_gaming_analysis.xlsx
@@ -487,22 +487,22 @@
         <v>46285</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>3601338</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>35551693</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>36576450</v>
       </c>
       <c r="E2" t="n">
         <v>208382110</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>237685605</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>70379895</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -511,10 +511,10 @@
         <v>10991490</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>7913221</v>
       </c>
       <c r="K2" t="n">
-        <v>219373600</v>
+        <v>611081802</v>
       </c>
     </row>
     <row r="3">
@@ -534,7 +534,7 @@
         <v>216744126</v>
       </c>
       <c r="F3" t="n">
-        <v>224469223</v>
+        <v>224469248</v>
       </c>
       <c r="G3" t="n">
         <v>60516979</v>
@@ -549,7 +549,7 @@
         <v>7510657</v>
       </c>
       <c r="K3" t="n">
-        <v>594594255</v>
+        <v>594594280</v>
       </c>
     </row>
     <row r="4">
@@ -9168,22 +9168,22 @@
         <v>46285</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>247569</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2928353</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2038071</v>
       </c>
       <c r="E2" t="n">
         <v>14221076</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>12919114</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>4708786</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -9192,10 +9192,10 @@
         <v>715640</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>728704</v>
       </c>
       <c r="K2" t="n">
-        <v>14936716</v>
+        <v>38507313</v>
       </c>
     </row>
     <row r="3">
@@ -9215,7 +9215,7 @@
         <v>4743263</v>
       </c>
       <c r="F3" t="n">
-        <v>8347252</v>
+        <v>8347277</v>
       </c>
       <c r="G3" t="n">
         <v>642600</v>
@@ -9230,7 +9230,7 @@
         <v>420192</v>
       </c>
       <c r="K3" t="n">
-        <v>16963048</v>
+        <v>16963073</v>
       </c>
     </row>
     <row r="4">
@@ -17848,21 +17848,33 @@
       <c r="A2" s="1" t="n">
         <v>46285</v>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>0.06874361695569814</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0.08236887621638722</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>0.05572085317191799</v>
+      </c>
       <c r="E2" s="2" t="n">
         <v>0.06824518669093042</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>0.05435379227109694</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.06690527173989105</v>
+      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
         <v>0.06510855216171783</v>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>0.09208690114935499</v>
+      </c>
       <c r="K2" s="2" t="n">
-        <v>0.06808802882388765</v>
+        <v>0.06301498894905727</v>
       </c>
     </row>
     <row r="3">
@@ -17882,7 +17894,7 @@
         <v>0.02188415938893772</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.03718662134808566</v>
+        <v>0.03718672858029978</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0.0106185075761961</v>
@@ -17895,7 +17907,7 @@
         <v>0.05594610431550795</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0.02852877883927755</v>
+        <v>0.02852881968524823</v>
       </c>
     </row>
     <row r="4">
@@ -26246,32 +26258,32 @@
         <v>46285</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-1</v>
+        <v>0.08858549460700482</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.03335303422830427</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1</v>
+        <v>0.004485305655987926</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>-0.05200454425422985</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1</v>
+        <v>0.2306729922153381</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>0.5655901153502181</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
         <v>0.02608325326799155</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.2622904956061224</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.6053302160863016</v>
+        <v>0.09938261827737471</v>
       </c>
     </row>
     <row r="3">
@@ -26291,7 +26303,7 @@
         <v>0.07104311570147237</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.2824596359472595</v>
+        <v>0.2824597787797176</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>-0.08246389845103475</v>
@@ -26304,7 +26316,7 @@
         <v>-0.3563374433577221</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0.1139180403821447</v>
+        <v>0.1139180872173617</v>
       </c>
     </row>
     <row r="4">
@@ -33729,32 +33741,32 @@
         <v>46285</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-1</v>
+        <v>1.951466380543634</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-1</v>
+        <v>0.447339598451217</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.2981119248627095</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>-0.3663476573970016</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.4602121720558833</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>0.1038749200597888</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
         <v>0.3916567490412961</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.003848157054020418</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.7374872058388652</v>
+        <v>-0.3232339470558728</v>
       </c>
     </row>
     <row r="3">
@@ -33774,7 +33786,7 @@
         <v>-0.7645204580808593</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-0.6535737949166487</v>
+        <v>-0.6535727573709837</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>-0.8838066083409352</v>
@@ -33787,7 +33799,7 @@
         <v>-0.4056337151570532</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>-0.7016844169475974</v>
+        <v>-0.7016839772925557</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Update NY gaming data - Thu Oct  1 17:56:35 UTC 2026
</commit_message>
<xml_diff>
--- a/ny_gaming_analysis.xlsx
+++ b/ny_gaming_analysis.xlsx
@@ -487,34 +487,34 @@
         <v>46292</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>3245265</v>
       </c>
       <c r="C2" t="n">
         <v>33450400</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>37726553</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>196194870</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>221260979</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>64794472</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>10286402</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>6391613</v>
       </c>
       <c r="K2" t="n">
-        <v>33450400</v>
+        <v>573350554</v>
       </c>
     </row>
     <row r="3">
@@ -9203,34 +9203,34 @@
         <v>46292</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>380853</v>
       </c>
       <c r="C2" t="n">
         <v>2799815</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>1308777.690000006</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>18137767</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>20111002</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>4300521</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>830090</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>718739.5399999998</v>
       </c>
       <c r="K2" t="n">
-        <v>2799815</v>
+        <v>48587565.23</v>
       </c>
     </row>
     <row r="3">
@@ -17918,19 +17918,33 @@
       <c r="A2" s="1" t="n">
         <v>46292</v>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>0.1173565178806661</v>
+      </c>
       <c r="C2" s="2" t="n">
         <v>0.08370049386554421</v>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>0.03469115479487367</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.09244771282755762</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.09089267385009626</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0.06637172689670193</v>
+      </c>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+      <c r="I2" s="2" t="n">
+        <v>0.08069779889994577</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0.1124504158809364</v>
+      </c>
       <c r="K2" s="2" t="n">
-        <v>0.08370049386554421</v>
+        <v>0.08474320795720379</v>
       </c>
     </row>
     <row r="3">
@@ -26347,32 +26361,32 @@
         <v>46292</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.01025046700468912</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>-0.07784786877201544</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.03620316414824376</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.0204366717917509</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1</v>
+        <v>0.08472810721003965</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>0.4251013249910285</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.04959407907131064</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.426962782511588</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.9392260489366314</v>
+        <v>0.04168495775689518</v>
       </c>
     </row>
     <row r="3">
@@ -33863,32 +33877,32 @@
         <v>46292</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-1</v>
+        <v>0.2957312820443032</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>-0.3446826966310018</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.4000764173023672</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.2182324179449213</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1</v>
+        <v>0.4643608634507477</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.04010598624526918</v>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.3206363392325169</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-1</v>
+        <v>-0.1559572494198775</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>-0.9442669616944011</v>
+        <v>-0.03281729895033214</v>
       </c>
     </row>
     <row r="3">

</xml_diff>